<commit_message>
Remove all non-essential spreadsheets, presentations, and reports with real client data to ensure total LGPD compliance, and anonymize sample.xlsx
</commit_message>
<xml_diff>
--- a/IceCream Co._ReportsAuto/optimareports-app/sample.xlsx
+++ b/IceCream Co._ReportsAuto/optimareports-app/sample.xlsx
@@ -16,551 +16,551 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="181">
-  <si>
-    <t>To see online:</t>
-  </si>
-  <si>
-    <t>www.yedda.tech</t>
-  </si>
-  <si>
-    <t>Company</t>
-  </si>
-  <si>
-    <t>DA07QUMX</t>
-  </si>
-  <si>
-    <t>Date Range</t>
-  </si>
-  <si>
-    <t>2026-04-01_2026-04-30</t>
-  </si>
-  <si>
-    <t>Time Range</t>
-  </si>
-  <si>
-    <t>00:00:00-23:59:59</t>
-  </si>
-  <si>
-    <t>Compare</t>
-  </si>
-  <si>
-    <t>None</t>
-  </si>
-  <si>
-    <t>Métricas</t>
-  </si>
-  <si>
-    <t>Total</t>
-  </si>
-  <si>
-    <t>48 Acanto</t>
-  </si>
-  <si>
-    <t>49 Arcos del Poniente</t>
-  </si>
-  <si>
-    <t>50 Citadina Escobedo</t>
-  </si>
-  <si>
-    <t>51 Concordia</t>
-  </si>
-  <si>
-    <t>52 Contry</t>
-  </si>
-  <si>
-    <t>53 Cumbres</t>
-  </si>
-  <si>
-    <t>54 El Jaral</t>
-  </si>
-  <si>
-    <t>55 Heberto Castillo</t>
-  </si>
-  <si>
-    <t>56 Israel Cavazos</t>
-  </si>
-  <si>
-    <t>57 Kune</t>
-  </si>
-  <si>
-    <t>58 La puerta</t>
-  </si>
-  <si>
-    <t>59 Las puentes</t>
-  </si>
-  <si>
-    <t>60 Las Torres</t>
-  </si>
-  <si>
-    <t>61 Rivera del Sol</t>
-  </si>
-  <si>
-    <t>62 Romulo Garza</t>
-  </si>
-  <si>
-    <t>63 San Jeronimo</t>
-  </si>
-  <si>
-    <t>65 Valle alto</t>
-  </si>
-  <si>
-    <t>Overview</t>
-  </si>
-  <si>
-    <t>Improving Customer Experience</t>
-  </si>
-  <si>
-    <t>Improving Operational Compliance</t>
-  </si>
-  <si>
-    <t>Reduce Costs</t>
-  </si>
-  <si>
-    <t>Total Notifications KBP</t>
-  </si>
-  <si>
-    <t>Total Service time</t>
-  </si>
-  <si>
-    <t>∑ Alerts of all types</t>
-  </si>
-  <si>
-    <t>Cashier Area</t>
-  </si>
-  <si>
-    <t>04:36</t>
-  </si>
-  <si>
-    <t>04:49</t>
-  </si>
-  <si>
-    <t>05:04</t>
-  </si>
-  <si>
-    <t>04:59</t>
-  </si>
-  <si>
-    <t>04:09</t>
-  </si>
-  <si>
-    <t>03:55</t>
-  </si>
-  <si>
-    <t>05:16</t>
-  </si>
-  <si>
-    <t>04:40</t>
-  </si>
-  <si>
-    <t>04:27</t>
-  </si>
-  <si>
-    <t>05:52</t>
-  </si>
-  <si>
-    <t>05:03</t>
-  </si>
-  <si>
-    <t>03:49</t>
-  </si>
-  <si>
-    <t>05:01</t>
-  </si>
-  <si>
-    <t>05:21</t>
-  </si>
-  <si>
-    <t>05:20</t>
-  </si>
-  <si>
-    <t>04:11</t>
-  </si>
-  <si>
-    <t>02:33</t>
-  </si>
-  <si>
-    <t>Less than 3min</t>
-  </si>
-  <si>
-    <t>3 to 5 minutes</t>
-  </si>
-  <si>
-    <t>For over 5 minutes</t>
-  </si>
-  <si>
-    <t>Ordering time</t>
-  </si>
-  <si>
-    <t>01:45</t>
-  </si>
-  <si>
-    <t>01:33</t>
-  </si>
-  <si>
-    <t>01:51</t>
-  </si>
-  <si>
-    <t>01:47</t>
-  </si>
-  <si>
-    <t>01:32</t>
-  </si>
-  <si>
-    <t>01:21</t>
-  </si>
-  <si>
-    <t>02:01</t>
-  </si>
-  <si>
-    <t>01:59</t>
-  </si>
-  <si>
-    <t>02:22</t>
-  </si>
-  <si>
-    <t>01:43</t>
-  </si>
-  <si>
-    <t>02:06</t>
-  </si>
-  <si>
-    <t>02:19</t>
-  </si>
-  <si>
-    <t>01:26</t>
-  </si>
-  <si>
-    <t>01:05</t>
-  </si>
-  <si>
-    <t>Less than 1 minutes</t>
-  </si>
-  <si>
-    <t>1 min to 2min</t>
-  </si>
-  <si>
-    <t>Over 2 minutes</t>
-  </si>
-  <si>
-    <t>Queuing Time</t>
-  </si>
-  <si>
-    <t>01:11</t>
-  </si>
-  <si>
-    <t>01:12</t>
-  </si>
-  <si>
-    <t>01:07</t>
-  </si>
-  <si>
-    <t>01:15</t>
-  </si>
-  <si>
-    <t>00:59</t>
-  </si>
-  <si>
-    <t>01:25</t>
-  </si>
-  <si>
-    <t>01:01</t>
-  </si>
-  <si>
-    <t>01:08</t>
-  </si>
-  <si>
-    <t>01:03</t>
-  </si>
-  <si>
-    <t>01:04</t>
-  </si>
-  <si>
-    <t>1min to 2min</t>
-  </si>
-  <si>
-    <t>Receiving Time</t>
-  </si>
-  <si>
-    <t>01:53</t>
-  </si>
-  <si>
-    <t>02:12</t>
-  </si>
-  <si>
-    <t>02:00</t>
-  </si>
-  <si>
-    <t>02:03</t>
-  </si>
-  <si>
-    <t>01:58</t>
-  </si>
-  <si>
-    <t>01:31</t>
-  </si>
-  <si>
-    <t>01:44</t>
-  </si>
-  <si>
-    <t>02:08</t>
-  </si>
-  <si>
-    <t>01:13</t>
-  </si>
-  <si>
-    <t>02:39</t>
-  </si>
-  <si>
-    <t>01:52</t>
-  </si>
-  <si>
-    <t>01:17</t>
-  </si>
-  <si>
-    <t>Total Alerts of Cashier Area</t>
-  </si>
-  <si>
-    <t>Cash around the cash counter</t>
-  </si>
-  <si>
-    <t>Cash drawer open and unattended for over 0 minute</t>
-  </si>
-  <si>
-    <t>Client not attended for over 1 minute</t>
-  </si>
-  <si>
-    <t>Counter dirty  for over 3 minutes</t>
-  </si>
-  <si>
-    <t>Manager does not deposit the partial cash withdrawal into the safe or electronic vault within 3 minutes</t>
-  </si>
-  <si>
-    <t>More than 3 people in line with only one register open</t>
-  </si>
-  <si>
-    <t>Personal taking cash without reporting it</t>
-  </si>
-  <si>
-    <t>Possible Theft</t>
-  </si>
-  <si>
-    <t>Receipt not given Counter</t>
-  </si>
-  <si>
-    <t>Receipt not printed Counter</t>
-  </si>
-  <si>
-    <t>Receive order for over 3 minutes</t>
-  </si>
-  <si>
-    <t>Staff outside the cash register area for over 1 minute</t>
-  </si>
-  <si>
-    <t>Staff putting money in their pockets</t>
-  </si>
-  <si>
-    <t>Staff using calculator/mobile phone near cashier</t>
-  </si>
-  <si>
-    <t>Staff using the customer’s bank card PIN pad</t>
-  </si>
-  <si>
-    <t>Staff using the manager’s card not the manager</t>
-  </si>
-  <si>
-    <t>Cam Check</t>
-  </si>
-  <si>
-    <t>Total Alerts of Cam Check</t>
-  </si>
-  <si>
-    <t>Angle Change</t>
-  </si>
-  <si>
-    <t>Blurry Image</t>
-  </si>
-  <si>
-    <t>Camera lagging</t>
-  </si>
-  <si>
-    <t>Can't connect to camera</t>
-  </si>
-  <si>
-    <t>Lost Connection</t>
-  </si>
-  <si>
-    <t>Obstructed camera</t>
-  </si>
-  <si>
-    <t>Time on camera differs real time</t>
-  </si>
-  <si>
-    <t>All Store</t>
-  </si>
-  <si>
-    <t>Traffic</t>
-  </si>
-  <si>
-    <t>Women</t>
-  </si>
-  <si>
-    <t>Couples</t>
-  </si>
-  <si>
-    <t>Total Alerts of All Store</t>
-  </si>
-  <si>
-    <t>Complaining customer</t>
-  </si>
-  <si>
-    <t>Dirty floor for over 3 minutes</t>
-  </si>
-  <si>
-    <t>Incomplete refrigerators (novelties)</t>
-  </si>
-  <si>
-    <t>Lost customer</t>
-  </si>
-  <si>
-    <t>More than 2 staff together inactive over 5 minutes</t>
-  </si>
-  <si>
-    <t>Personal playing or fighting</t>
-  </si>
-  <si>
-    <t>Refrigerator doors open for more than 1 minute</t>
-  </si>
-  <si>
-    <t>Staff without caps</t>
-  </si>
-  <si>
-    <t>Staff without uniform</t>
-  </si>
-  <si>
-    <t>Store close sooner</t>
-  </si>
-  <si>
-    <t>Store open late</t>
-  </si>
-  <si>
-    <t>Delivery</t>
-  </si>
-  <si>
-    <t>Delivery waiting time</t>
-  </si>
-  <si>
-    <t>02:24</t>
-  </si>
-  <si>
-    <t>01:36</t>
-  </si>
-  <si>
-    <t>03:53</t>
-  </si>
-  <si>
-    <t>02:10</t>
-  </si>
-  <si>
-    <t>03:09</t>
-  </si>
-  <si>
-    <t>03:02</t>
-  </si>
-  <si>
-    <t>03:33</t>
-  </si>
-  <si>
-    <t>00:30</t>
-  </si>
-  <si>
-    <t>02:54</t>
-  </si>
-  <si>
-    <t>02:25</t>
-  </si>
-  <si>
-    <t>01:54</t>
-  </si>
-  <si>
-    <t>02:23</t>
-  </si>
-  <si>
-    <t>01:20</t>
-  </si>
-  <si>
-    <t>02:09</t>
-  </si>
-  <si>
-    <t>Less than 2 min</t>
-  </si>
-  <si>
-    <t>2:00 - 3:00</t>
-  </si>
-  <si>
-    <t>More than 3 min</t>
-  </si>
-  <si>
-    <t>Total Alerts of Delivery</t>
-  </si>
-  <si>
-    <t>Check packaging</t>
-  </si>
-  <si>
-    <t>Delivery guy waiting more than 1 minute</t>
-  </si>
-  <si>
-    <t>Delivery man putting product in clothes</t>
-  </si>
-  <si>
-    <t>Package closed</t>
-  </si>
-  <si>
-    <t>Drive Thru</t>
-  </si>
-  <si>
-    <t>Total Alerts Drive Thru</t>
-  </si>
-  <si>
-    <t>[D] Cash around the cash counter</t>
-  </si>
-  <si>
-    <t>[D] Cash drawer open and unattended</t>
-  </si>
-  <si>
-    <t>[D] Manager does not deposit the partial cash withdrawal into the safe or electronic vault within 3 minutes</t>
-  </si>
-  <si>
-    <t>[D] Other possible theft</t>
-  </si>
-  <si>
-    <t>[D] Receipt not delivered</t>
-  </si>
-  <si>
-    <t>[D] Receipt not printed</t>
-  </si>
-  <si>
-    <t>[D] Receipts around the cash register</t>
-  </si>
-  <si>
-    <t>[D] Staff outside the cash register area for over 1 minute</t>
-  </si>
-  <si>
-    <t>[D] Staff storing cash in their pockets</t>
-  </si>
-  <si>
-    <t>[D] Staff taking cash without reporting it Counter</t>
-  </si>
-  <si>
-    <t>[D] Staff using calculator or mobile phone near the cash register (not manager)</t>
-  </si>
-  <si>
-    <t>[D] Staff using the customer’s bank card PIN pad</t>
-  </si>
-  <si>
-    <t>[D] Staff using the manager’s card not the manager</t>
-  </si>
-</sst>
+<ns0:sst xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="181">
+  <ns0:si>
+    <ns0:t>To see online:</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>www.optimareports.ai</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Company</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Restaurant Co.</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Date Range</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>2026-04-01_2026-04-30</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Time Range</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>00:00:00-23:59:59</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Compare</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>None</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Métricas</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Total</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Store 01</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Store 02</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Store 03</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Store 04</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Store 05</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Store 06</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Store 07</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Store 08</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Store 09</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Store 10</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Store 11</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Store 12</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Store 13</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Store 14</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Store 15</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Store 16</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Store 17</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Overview</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Improving Customer Experience</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Improving Operational Compliance</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Reduce Costs</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Total Notifications KBP</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Total Service time</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>∑ Alerts of all types</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Cashier Area</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>04:36</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>04:49</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>05:04</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>04:59</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>04:09</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>03:55</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>05:16</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>04:40</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>04:27</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>05:52</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>05:03</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>03:49</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>05:01</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>05:21</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>05:20</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>04:11</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>02:33</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Less than 3min</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>3 to 5 minutes</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>For over 5 minutes</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Ordering time</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>01:45</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>01:33</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>01:51</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>01:47</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>01:32</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>01:21</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>02:01</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>01:59</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>02:22</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>01:43</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>02:06</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>02:19</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>01:26</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>01:05</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Less than 1 minutes</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>1 min to 2min</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Over 2 minutes</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Queuing Time</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>01:11</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>01:12</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>01:07</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>01:15</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>00:59</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>01:25</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>01:01</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>01:08</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>01:03</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>01:04</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>1min to 2min</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Receiving Time</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>01:53</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>02:12</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>02:00</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>02:03</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>01:58</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>01:31</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>01:44</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>02:08</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>01:13</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>02:39</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>01:52</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>01:17</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Total Alerts of Cashier Area</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Cash around the cash counter</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Cash drawer open and unattended for over 0 minute</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Client not attended for over 1 minute</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Counter dirty  for over 3 minutes</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Manager does not deposit the partial cash withdrawal into the safe or electronic vault within 3 minutes</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>More than 3 people in line with only one register open</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Personal taking cash without reporting it</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Possible Theft</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Receipt not given Counter</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Receipt not printed Counter</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Receive order for over 3 minutes</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Staff outside the cash register area for over 1 minute</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Staff putting money in their pockets</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Staff using calculator/mobile phone near cashier</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Staff using the customer’s bank card PIN pad</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Staff using the manager’s card not the manager</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Cam Check</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Total Alerts of Cam Check</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Angle Change</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Blurry Image</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Camera lagging</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Can't connect to camera</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Lost Connection</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Obstructed camera</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Time on camera differs real time</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>All Store</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Traffic</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Women</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Couples</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Total Alerts of All Store</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Complaining customer</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Dirty floor for over 3 minutes</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Incomplete refrigerators (novelties)</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Lost customer</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>More than 2 staff together inactive over 5 minutes</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Personal playing or fighting</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Refrigerator doors open for more than 1 minute</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Staff without caps</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Staff without uniform</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Store close sooner</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Store open late</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Delivery</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Delivery waiting time</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>02:24</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>01:36</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>03:53</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>02:10</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>03:09</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>03:02</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>03:33</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>00:30</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>02:54</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>02:25</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>01:54</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>02:23</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>01:20</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>02:09</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Less than 2 min</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>2:00 - 3:00</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>More than 3 min</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Total Alerts of Delivery</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Check packaging</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Delivery guy waiting more than 1 minute</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Delivery man putting product in clothes</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Package closed</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Drive Thru</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Total Alerts Drive Thru</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>[D] Cash around the cash counter</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>[D] Cash drawer open and unattended</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>[D] Manager does not deposit the partial cash withdrawal into the safe or electronic vault within 3 minutes</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>[D] Other possible theft</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>[D] Receipt not delivered</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>[D] Receipt not printed</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>[D] Receipts around the cash register</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>[D] Staff outside the cash register area for over 1 minute</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>[D] Staff storing cash in their pockets</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>[D] Staff taking cash without reporting it Counter</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>[D] Staff using calculator or mobile phone near the cash register (not manager)</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>[D] Staff using the customer’s bank card PIN pad</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>[D] Staff using the manager’s card not the manager</ns0:t>
+  </ns0:si>
+</ns0:sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>